<commit_message>
Excel de precios: Patrocinio -> Beca del Fondo (15 celdas, Ley 1480; sin tocar numeros ni formulas)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7C5dx3NvDfXiv3CfhPMa
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/Tabla Precios Heiiu 2026 INTERNO (1).xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/Tabla Precios Heiiu 2026 INTERNO (1).xlsx
@@ -525,13 +525,15 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CONTADO — Patrocinio 45% — $4.782.800</t>
-        </is>
-      </c>
-    </row>
+          <t>CONTADO — Beca del Fondo 45% — $4.782.800</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -542,7 +544,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $8,696,000 | Patrocinio: 35% | Precio con patrocinio: $5,652,400 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $8,696,000 | Beca del Fondo: 35% | Precio con beca del Fondo: $5,652,400 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -729,6 +731,7 @@
         <v>153900</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -739,7 +742,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $8,696,000 | Patrocinio: 35% | Precio con patrocinio: $5,652,400 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $8,696,000 | Beca del Fondo: 35% | Precio con beca del Fondo: $5,652,400 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -1020,13 +1023,15 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CONTADO — Patrocinio 35% — $4.615.000</t>
-        </is>
-      </c>
-    </row>
+          <t>CONTADO — Beca del Fondo 35% — $4.615.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1037,7 +1042,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $7,100,000 | Patrocinio: 25% | Precio con patrocinio: $5,325,000 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $7,100,000 | Beca del Fondo: 25% | Precio con beca del Fondo: $5,325,000 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -1224,6 +1229,7 @@
         <v>134905</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1234,7 +1240,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $7,100,000 | Patrocinio: 25% | Precio con patrocinio: $5,325,000 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $7,100,000 | Beca del Fondo: 25% | Precio con beca del Fondo: $5,325,000 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -1515,13 +1521,15 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CONTADO — Patrocinio 25% — $3.888.750</t>
-        </is>
-      </c>
-    </row>
+          <t>CONTADO — Beca del Fondo 25% — $3.888.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1532,7 +1540,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $5,185,000 | Patrocinio: 15% | Precio con patrocinio: $4,407,250 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $5,185,000 | Beca del Fondo: 15% | Precio con beca del Fondo: $4,407,250 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -1696,6 +1704,7 @@
         <v>73317</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1706,7 +1715,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $5,185,000 | Patrocinio: 15% | Precio con patrocinio: $4,407,250 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $5,185,000 | Beca del Fondo: 15% | Precio con beca del Fondo: $4,407,250 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -1941,6 +1950,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1955,6 +1965,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -1965,7 +1976,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $1,596,000 | Patrocinio: 10% | Precio con patrocinio: $1,436,400 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $1,596,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $1,436,400 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -2123,6 +2134,7 @@
         <v>36925</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
@@ -2137,6 +2149,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -2147,7 +2160,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $1,915,000 | Patrocinio: 10% | Precio con patrocinio: $1,723,500 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $1,915,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $1,723,500 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -2271,6 +2284,7 @@
         <v>20794</v>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -2281,7 +2295,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $1,915,000 | Patrocinio: 10% | Precio con patrocinio: $1,723,500 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $1,915,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $1,723,500 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -2465,6 +2479,7 @@
         <v>49126</v>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
@@ -2479,6 +2494,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
@@ -2489,7 +2505,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $2,842,000 | Patrocinio: 10% | Precio con patrocinio: $2,557,800 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $2,842,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $2,557,800 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -2633,6 +2649,7 @@
         <v>40662</v>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
@@ -2643,7 +2660,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $2,842,000 | Patrocinio: 10% | Precio con patrocinio: $2,557,800 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $2,842,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $2,557,800 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>
@@ -2827,6 +2844,7 @@
         <v>103569</v>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
@@ -2841,6 +2859,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
@@ -2851,7 +2870,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Precio full: $2,343,000 | Patrocinio: 10% | Precio con patrocinio: $2,108,700 | Tasa crédito: 1.9% mensual</t>
+          <t>Precio full: $2,343,000 | Beca del Fondo: 10% | Precio con beca del Fondo: $2,108,700 | Tasa crédito: 1.9% mensual</t>
         </is>
       </c>
     </row>

</xml_diff>